<commit_message>
n8n board refresh 2026-09-29T17:40:29Z
</commit_message>
<xml_diff>
--- a/app/reports/GAM_research.xlsx
+++ b/app/reports/GAM_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-29 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>64.52</v>
+        <v>63.83</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05184000015258789</v>
+        <v>0.05293000221252441</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>23832110.10539368</v>
+        <v>23832112.04762651</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>64.52</v>
+        <v>63.83</v>
       </c>
     </row>
     <row r="38">
@@ -1508,14 +1508,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>1537647744</v>
+        <v>1521203712</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>4.05</v>
+        <v>4</v>
       </c>
       <c r="E5" s="31" t="n"/>
       <c r="F5" s="31" t="n">
-        <v>70.5</v>
+        <v>69.98</v>
       </c>
     </row>
     <row r="6">
@@ -1530,16 +1530,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>3331813120</v>
+        <v>3238119168</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>33.173145</v>
+        <v>32.240284</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>20.541</v>
+        <v>20.523</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>5.334</v>
+        <v>5.329</v>
       </c>
     </row>
     <row r="7">
@@ -1555,13 +1555,13 @@
       </c>
       <c r="C7" s="32" t="n"/>
       <c r="D7" s="33" t="n">
-        <v>7.558981</v>
+        <v>7.402815</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>46.582</v>
+        <v>45.617</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>38.674</v>
+        <v>37.872</v>
       </c>
     </row>
     <row r="8">
@@ -1576,14 +1576,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>2556645888</v>
+        <v>2507660800</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>13.090033</v>
+        <v>12.839229</v>
       </c>
       <c r="E8" s="33" t="n"/>
       <c r="F8" s="33" t="n">
-        <v>5.557</v>
+        <v>5.524</v>
       </c>
     </row>
     <row r="9">
@@ -1598,10 +1598,10 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>1033597952</v>
+        <v>1040677312</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>8.377049</v>
+        <v>8.434426</v>
       </c>
       <c r="E9" s="33" t="n"/>
       <c r="F9" s="33" t="n"/>
@@ -1618,14 +1618,14 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>1073908864</v>
+        <v>1065466176</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>18.346155</v>
+        <v>18.201923</v>
       </c>
       <c r="E10" s="33" t="n"/>
       <c r="F10" s="33" t="n">
-        <v>8.561</v>
+        <v>8.534000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1640,14 +1640,14 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>2393373696</v>
+        <v>2291850496</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>10.461847</v>
+        <v>10.018072</v>
       </c>
       <c r="E11" s="33" t="n"/>
       <c r="F11" s="33" t="n">
-        <v>10.203</v>
+        <v>10.163</v>
       </c>
     </row>
     <row r="12">
@@ -1662,14 +1662,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>1201862144</v>
+        <v>1194292736</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>20.710144</v>
+        <v>20.57971</v>
       </c>
       <c r="E12" s="33" t="n"/>
       <c r="F12" s="33" t="n">
-        <v>8.356</v>
+        <v>8.326000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1684,12 +1684,12 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>876390400</v>
+        <v>877860864</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n"/>
       <c r="F13" s="33" t="n">
-        <v>3.338</v>
+        <v>3.331</v>
       </c>
     </row>
     <row r="15">

</xml_diff>